<commit_message>
Fixed pdf invoice template
</commit_message>
<xml_diff>
--- a/Trip_Data_Store/uhc_sample1.xlsx
+++ b/Trip_Data_Store/uhc_sample1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kshema/python/Four-Line-Travels/Trip_Data_Store/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EA2929D1-4D0F-8B41-8F29-B5D265CF1166}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1B39060-EE19-D044-BB55-7D8375450650}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20840" xr2:uid="{DD45487B-C340-664F-BE75-A1545FFE3B33}"/>
   </bookViews>
@@ -56,9 +56,6 @@
     <t>Facility Name</t>
   </si>
   <si>
-    <t>Patient Address</t>
-  </si>
-  <si>
     <t>John Smith</t>
   </si>
   <si>
@@ -72,6 +69,9 @@
   </si>
   <si>
     <t>152 Stevens Avenue, Jersey City, NJ 07305</t>
+  </si>
+  <si>
+    <t>Destination Address</t>
   </si>
 </sst>
 </file>
@@ -489,30 +489,30 @@
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>7</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>8</v>
       </c>
       <c r="C2" s="2">
         <v>123456789</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E2" s="3">
         <v>46084</v>
       </c>
       <c r="F2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>10</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>